<commit_message>
fix(legacy-bridge): excel.ts model.media + hyperlink/Date guard + escapeMd \r 处理(round 2)
</commit_message>
<xml_diff>
--- a/tests/fixtures/legacy-bridge/excel-test-cases.xlsx
+++ b/tests/fixtures/legacy-bridge/excel-test-cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>ID</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>返回原响应不重复扣款</t>
+  </si>
+  <si>
+    <t>TC-004</t>
+  </si>
+  <si>
+    <t>点击此链接</t>
+  </si>
+  <si>
+    <t>点链接</t>
   </si>
   <si>
     <t>模块</t>
@@ -122,8 +131,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -522,7 +532,24 @@
         <v>15</v>
       </c>
     </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1">
+        <v>46037.33333333333</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -535,35 +562,35 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>